<commit_message>
Modification Tableau de synthèse
</commit_message>
<xml_diff>
--- a/Documents/Tableau_de_synthèse_E5_Benjamin_MAIRE.xlsx
+++ b/Documents/Tableau_de_synthèse_E5_Benjamin_MAIRE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\source\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\source\Portfolio\benjaminmaire.github.io\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CF4EDA4-6D40-40A9-B596-5140B0FB0966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64075677-E413-4F81-B546-22BDAFDB97DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="44">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -119,55 +119,62 @@
     <t>Centre de formation : CFA ITIS</t>
   </si>
   <si>
-    <t>01/03/2025 au 20/03/2026</t>
-  </si>
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>Application Mobile de gestion d'évènements EvenixMobile</t>
-  </si>
-  <si>
-    <t>Application Web de gestion d'évènements Evenix</t>
-  </si>
-  <si>
-    <t>Logiciel de gestion d'inventaire Pandore</t>
-  </si>
-  <si>
-    <t>Logiciel de création de commandes Socaphi</t>
-  </si>
-  <si>
     <t>04/01/2025 au 31/03/2025</t>
   </si>
   <si>
     <t>02/04/2025 au 30/05/2025</t>
   </si>
   <si>
-    <t>Application mobile de gestion d'inventaire Go/NoGo</t>
-  </si>
-  <si>
-    <t>Applicaiton mobile de lecture de QR code et d'écriture dans une puce RFID</t>
-  </si>
-  <si>
-    <t>Configuration de postes clients et élaboration de la documentation technique d'exploitation</t>
-  </si>
-  <si>
     <t>☑ SLAM</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Adresse URL du portfolio : </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="18"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>A compléter</t>
-    </r>
+    <t>Adresse URL du portfolio : https://benjaminmaire.github.io/</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Application mobile de gestion d'inventaire - Go/NoGo</t>
+  </si>
+  <si>
+    <t>Configuration de postes clients et élaboration de la documentation technique d'installation</t>
+  </si>
+  <si>
+    <t>Logiciel de création de commandes - Socaphi</t>
+  </si>
+  <si>
+    <t>Logiciel de gestion d'inventaire - Pandore</t>
+  </si>
+  <si>
+    <t>Application Web de gestion d'évènements - Evenix</t>
+  </si>
+  <si>
+    <t>Application Mobile de gestion d'évènements - EvenixMobile</t>
+  </si>
+  <si>
+    <t>02/09/2024 au 02/09/2026</t>
+  </si>
+  <si>
+    <t>02/09/2025 au 29/10/2025</t>
+  </si>
+  <si>
+    <t>03/11/2025 au 15/12/2025</t>
+  </si>
+  <si>
+    <t>01/03/2025 au 17/12/2025</t>
+  </si>
+  <si>
+    <t>07/01/2025 au 18/03/2026</t>
+  </si>
+  <si>
+    <t>Application mobile de lecture de QR code et d'écriture dans une puce RFID - BarcoTag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réalisation d'un Portfolio
+</t>
+  </si>
+  <si>
+    <t>01/03/2025 au 31/05/2025</t>
   </si>
 </sst>
 </file>
@@ -177,7 +184,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -239,18 +246,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="16"/>
-      <name val="Marlett"/>
-      <charset val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -651,7 +646,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -719,18 +714,54 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -753,45 +784,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1103,66 +1095,66 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AQ81"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" style="1" customWidth="1"/>
-    <col min="3" max="8" width="18.6640625" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.44140625" customWidth="1"/>
-    <col min="44" max="16384" width="10.88671875" style="1"/>
+    <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.42578125" customWidth="1"/>
+    <col min="44" max="16384" width="10.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="26"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
+      <c r="H1" s="27"/>
+    </row>
+    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-    </row>
-    <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+    </row>
+    <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="33" t="s">
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="28"/>
-      <c r="H3" s="34"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="46"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="30" t="s">
+    <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="32"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="44"/>
       <c r="F4" s="14" t="s">
         <v>8</v>
       </c>
@@ -1170,26 +1162,26 @@
         <v>15</v>
       </c>
       <c r="H4" s="21" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="45" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="46"/>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="46"/>
-      <c r="G5" s="46"/>
-      <c r="H5" s="47"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="35" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="43" t="s">
+      <c r="B6" s="34" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1211,9 +1203,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="36"/>
-      <c r="B7" s="44"/>
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="26"/>
+      <c r="B7" s="35"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1268,17 +1260,17 @@
       <c r="AP7"/>
       <c r="AQ7"/>
     </row>
-    <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="37" t="s">
+    <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A8" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="38"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="38"/>
-      <c r="G8" s="38"/>
-      <c r="H8" s="39"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1315,25 +1307,31 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="H9" s="25"/>
+        <v>39</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="23" t="s">
+        <v>29</v>
+      </c>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1370,26 +1368,28 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" s="25" t="s">
-        <v>26</v>
+        <v>40</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>29</v>
       </c>
       <c r="I10"/>
       <c r="J10"/>
@@ -1427,15 +1427,23 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
-      <c r="B11" s="10"/>
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>43</v>
+      </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
+      <c r="E11" s="16" t="s">
+        <v>29</v>
+      </c>
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
-      <c r="H11" s="24"/>
+      <c r="H11" s="23" t="s">
+        <v>29</v>
+      </c>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1472,7 +1480,7 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="11"/>
       <c r="B12" s="10"/>
       <c r="C12" s="16"/>
@@ -1480,7 +1488,7 @@
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
       <c r="G12" s="16"/>
-      <c r="H12" s="24"/>
+      <c r="H12" s="23"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1517,7 +1525,7 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="11"/>
       <c r="B13" s="10"/>
       <c r="C13" s="16"/>
@@ -1525,7 +1533,7 @@
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
-      <c r="H13" s="24"/>
+      <c r="H13" s="23"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1562,7 +1570,7 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="11"/>
       <c r="B14" s="10"/>
       <c r="C14" s="16"/>
@@ -1570,7 +1578,7 @@
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
-      <c r="H14" s="24"/>
+      <c r="H14" s="23"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1607,7 +1615,7 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="11"/>
       <c r="B15" s="10"/>
       <c r="C15" s="16"/>
@@ -1615,7 +1623,7 @@
       <c r="E15" s="16"/>
       <c r="F15" s="16"/>
       <c r="G15" s="16"/>
-      <c r="H15" s="24"/>
+      <c r="H15" s="23"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1652,7 +1660,7 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="11"/>
       <c r="B16" s="10"/>
       <c r="C16" s="16"/>
@@ -1660,7 +1668,7 @@
       <c r="E16" s="16"/>
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
-      <c r="H16" s="24"/>
+      <c r="H16" s="23"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1697,7 +1705,7 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="11"/>
       <c r="B17" s="10"/>
       <c r="C17" s="16"/>
@@ -1705,7 +1713,7 @@
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
       <c r="G17" s="16"/>
-      <c r="H17" s="24"/>
+      <c r="H17" s="23"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1742,7 +1750,7 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="11"/>
       <c r="B18" s="10"/>
       <c r="C18" s="16"/>
@@ -1750,7 +1758,7 @@
       <c r="E18" s="16"/>
       <c r="F18" s="16"/>
       <c r="G18" s="16"/>
-      <c r="H18" s="24"/>
+      <c r="H18" s="23"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1787,17 +1795,17 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A19" s="40" t="s">
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A19" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="41"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="41"/>
-      <c r="E19" s="41"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="41"/>
-      <c r="H19" s="42"/>
+      <c r="B19" s="32"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="33"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1834,23 +1842,23 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="H20" s="25"/>
+        <v>25</v>
+      </c>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="H20" s="23"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1887,25 +1895,27 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B21" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="C21" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="D21" s="23"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="G21" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="H21" s="25"/>
+      <c r="C21" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G21" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="H21" s="23"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1942,7 +1952,7 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="11"/>
       <c r="B22" s="10"/>
       <c r="C22" s="17"/>
@@ -1987,7 +1997,7 @@
       <c r="AP22"/>
       <c r="AQ22"/>
     </row>
-    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="11"/>
       <c r="B23" s="10"/>
       <c r="C23" s="17"/>
@@ -2032,7 +2042,7 @@
       <c r="AP23"/>
       <c r="AQ23"/>
     </row>
-    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="11"/>
       <c r="B24" s="10"/>
       <c r="C24" s="17"/>
@@ -2077,7 +2087,7 @@
       <c r="AP24"/>
       <c r="AQ24"/>
     </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="11"/>
       <c r="B25" s="10"/>
       <c r="C25" s="17"/>
@@ -2122,7 +2132,7 @@
       <c r="AP25"/>
       <c r="AQ25"/>
     </row>
-    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="11"/>
       <c r="B26" s="10"/>
       <c r="C26" s="17"/>
@@ -2167,17 +2177,17 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A27" s="40" t="s">
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+      <c r="A27" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="41"/>
-      <c r="C27" s="41"/>
-      <c r="D27" s="41"/>
-      <c r="E27" s="41"/>
-      <c r="F27" s="41"/>
-      <c r="G27" s="41"/>
-      <c r="H27" s="42"/>
+      <c r="B27" s="32"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="33"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2214,23 +2224,27 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B28" s="10"/>
-      <c r="C28" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="D28" s="23"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="G28" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="H28" s="25"/>
+        <v>30</v>
+      </c>
+      <c r="B28" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G28" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="H28" s="23"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2267,22 +2281,26 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B29" s="10"/>
-      <c r="C29" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="H29" s="25" t="s">
-        <v>26</v>
+        <v>41</v>
+      </c>
+      <c r="B29" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D29" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="H29" s="23" t="s">
+        <v>29</v>
       </c>
       <c r="I29"/>
       <c r="J29"/>
@@ -2320,21 +2338,23 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B30" s="10"/>
-      <c r="C30" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="D30" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="E30" s="23"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="23" t="s">
-        <v>26</v>
+        <v>31</v>
+      </c>
+      <c r="B30" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D30" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16" t="s">
+        <v>29</v>
       </c>
       <c r="H30" s="18"/>
       <c r="I30"/>
@@ -2373,7 +2393,7 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="11"/>
       <c r="B31" s="10"/>
       <c r="C31" s="17"/>
@@ -2418,7 +2438,7 @@
       <c r="AP31"/>
       <c r="AQ31"/>
     </row>
-    <row r="32" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="11"/>
       <c r="B32" s="10"/>
       <c r="C32" s="17"/>
@@ -2463,7 +2483,7 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="11"/>
       <c r="B33" s="10"/>
       <c r="C33" s="17"/>
@@ -2508,7 +2528,7 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="12"/>
       <c r="B34" s="13"/>
       <c r="C34" s="19"/>
@@ -2553,7 +2573,7 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:43" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A35" s="5"/>
       <c r="B35" s="3"/>
       <c r="C35" s="4"/>
@@ -2598,54 +2618,59 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="49" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="50" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="51" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="52" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="53" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="54" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="55" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="56" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="57" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="58" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="59" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="60" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="61" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="62" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="63" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="64" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="65" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="66" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="67" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="68" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="69" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="70" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="71" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="72" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="73" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="74" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="75" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="76" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="77" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="78" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="79" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="80" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="50" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="51" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="52" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="53" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="54" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="59" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="60" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="61" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="62" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="63" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="64" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="65" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="66" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="67" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="68" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="69" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="70" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="71" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="72" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="73" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="74" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="75" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="76" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="77" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="78" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="79" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="80" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="81" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2653,16 +2678,11 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="48" orientation="portrait"/>
+  <pageSetup paperSize="9" scale="48" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajout lien linkedin et documentations
</commit_message>
<xml_diff>
--- a/Documents/Tableau_de_synthèse_E5_Benjamin_MAIRE.xlsx
+++ b/Documents/Tableau_de_synthèse_E5_Benjamin_MAIRE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\source\Portfolio\benjaminmaire.github.io\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64075677-E413-4F81-B546-22BDAFDB97DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68DCABB7-AB03-4931-B2CD-6BE4E5C02FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="44">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -134,24 +134,6 @@
     <t>X</t>
   </si>
   <si>
-    <t>Application mobile de gestion d'inventaire - Go/NoGo</t>
-  </si>
-  <si>
-    <t>Configuration de postes clients et élaboration de la documentation technique d'installation</t>
-  </si>
-  <si>
-    <t>Logiciel de création de commandes - Socaphi</t>
-  </si>
-  <si>
-    <t>Logiciel de gestion d'inventaire - Pandore</t>
-  </si>
-  <si>
-    <t>Application Web de gestion d'évènements - Evenix</t>
-  </si>
-  <si>
-    <t>Application Mobile de gestion d'évènements - EvenixMobile</t>
-  </si>
-  <si>
     <t>02/09/2024 au 02/09/2026</t>
   </si>
   <si>
@@ -164,17 +146,42 @@
     <t>01/03/2025 au 17/12/2025</t>
   </si>
   <si>
-    <t>07/01/2025 au 18/03/2026</t>
-  </si>
-  <si>
-    <t>Application mobile de lecture de QR code et d'écriture dans une puce RFID - BarcoTag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réalisation d'un Portfolio
-</t>
-  </si>
-  <si>
     <t>01/03/2025 au 31/05/2025</t>
+  </si>
+  <si>
+    <t>Logiciel de gestion d'inventaire - Pandore (BARCODIS) Documents : code source VB.NET, documentation utilisateur</t>
+  </si>
+  <si>
+    <t>Logiciel de création de commandes - LegitrackCore (Socaphi)
+Documents : code source VB.NET</t>
+  </si>
+  <si>
+    <t>Application mobile de contrôle logistique - Go/NoGo (Safran)
+Documents : code source Android, documentation utilisateur</t>
+  </si>
+  <si>
+    <t>Application mobile RFID &amp; QR Code - BarcoTag (Continental)
+Documents : code source Android, documentation utilisateur</t>
+  </si>
+  <si>
+    <t>Configuration de postes clients et documentation 
+technique d'installation (BARCODIS)
+Documents : documentation technique d'installation</t>
+  </si>
+  <si>
+    <t>Réalisation d'un Portfolio professionnel BTS SIO 
+Documents : site en ligne sur benjaminmaire.github.io</t>
+  </si>
+  <si>
+    <t>Application Web de gestion d'évènements - Evenix
+Documents : code source GitHub, API Swagger UI, documentation technique, documentation utilisateur
+Production : application déployée sur evenix.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Application Mobile de gestion d'évènements - EvenixMobile Documents : code source GitHub, application testée iOS &amp; Android, documentation technique, documentation utilisateur </t>
+  </si>
+  <si>
+    <t>07/01/2026 au 18/03/2026</t>
   </si>
 </sst>
 </file>
@@ -255,7 +262,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -265,388 +272,42 @@
     </border>
     <border>
       <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border diagonalDown="1">
-      <left style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
+      <left style="thin">
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
+        <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
+      <top style="thin">
+        <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal style="thin">
         <color theme="2" tint="-0.749992370372631"/>
       </diagonal>
-    </border>
-    <border diagonalDown="1">
-      <left style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </diagonal>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -663,128 +324,47 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1105,123 +685,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27" t="s">
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="27"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="H1" s="14"/>
+    </row>
+    <row r="2" spans="1:43" ht="41.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
     </row>
     <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="45" t="s">
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="40"/>
-      <c r="H3" s="46"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="43"/>
-      <c r="C4" s="43"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="14" t="s">
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="21" t="s">
+      <c r="H4" s="11" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="36" t="s">
+    <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="38"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="12" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="26"/>
-      <c r="B7" s="35"/>
-      <c r="C7" s="8" t="s">
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="16"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="13" t="s">
         <v>14</v>
       </c>
       <c r="I7"/>
@@ -1261,16 +841,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="30"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1307,29 +887,29 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="G9" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="H9" s="23" t="s">
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="72.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="7" t="s">
         <v>29</v>
       </c>
       <c r="I9"/>
@@ -1368,27 +948,27 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="H10" s="23" t="s">
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="65.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="7" t="s">
         <v>29</v>
       </c>
       <c r="I10"/>
@@ -1427,21 +1007,21 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="B11" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="23" t="s">
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7" t="s">
         <v>29</v>
       </c>
       <c r="I11"/>
@@ -1481,14 +1061,14 @@
       <c r="AQ11"/>
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="11"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="23"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1526,14 +1106,14 @@
       <c r="AQ12"/>
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="11"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="23"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1571,14 +1151,14 @@
       <c r="AQ13"/>
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="11"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="23"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1616,14 +1196,14 @@
       <c r="AQ14"/>
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="11"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="23"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1661,14 +1241,14 @@
       <c r="AQ15"/>
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="11"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="23"/>
+      <c r="A16" s="6"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1706,14 +1286,14 @@
       <c r="AQ16"/>
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="11"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="23"/>
+      <c r="A17" s="6"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1751,14 +1331,14 @@
       <c r="AQ17"/>
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="11"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="23"/>
+      <c r="A18" s="6"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1796,16 +1376,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="31" t="s">
+      <c r="A19" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="32"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="33"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1842,23 +1422,25 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B20" s="22" t="s">
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="H20" s="23"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1895,27 +1477,27 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B21" s="22" t="s">
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="D21" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="G21" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="H21" s="23"/>
+      <c r="C21" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1953,14 +1535,14 @@
       <c r="AQ21"/>
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="11"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="18"/>
+      <c r="A22" s="6"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -1998,14 +1580,14 @@
       <c r="AQ22"/>
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="11"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="18"/>
+      <c r="A23" s="6"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -2043,14 +1625,14 @@
       <c r="AQ23"/>
     </row>
     <row r="24" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="11"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="18"/>
+      <c r="A24" s="6"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -2088,14 +1670,14 @@
       <c r="AQ24"/>
     </row>
     <row r="25" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="11"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="18"/>
+      <c r="A25" s="6"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2133,14 +1715,14 @@
       <c r="AQ25"/>
     </row>
     <row r="26" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="11"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="18"/>
+      <c r="A26" s="6"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2178,16 +1760,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A27" s="31" t="s">
+      <c r="A27" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="32"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
-      <c r="H27" s="33"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2224,27 +1806,27 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" s="22" t="s">
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="G28" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="H28" s="23"/>
+      <c r="B28" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2281,25 +1863,25 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B29" s="22" t="s">
+    <row r="29" spans="1:43" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C29" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="D29" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="H29" s="23" t="s">
+      <c r="B29" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H29" s="7" t="s">
         <v>29</v>
       </c>
       <c r="I29"/>
@@ -2338,25 +1920,27 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="C30" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="D30" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="H30" s="18"/>
+    <row r="30" spans="1:43" s="2" customFormat="1" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2394,14 +1978,14 @@
       <c r="AQ30"/>
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="11"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="18"/>
+      <c r="A31" s="6"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
+      <c r="G31" s="9"/>
+      <c r="H31" s="9"/>
       <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
@@ -2439,14 +2023,14 @@
       <c r="AQ31"/>
     </row>
     <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="11"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
-      <c r="G32" s="17"/>
-      <c r="H32" s="18"/>
+      <c r="A32" s="6"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
       <c r="I32"/>
       <c r="J32"/>
       <c r="K32"/>
@@ -2484,14 +2068,14 @@
       <c r="AQ32"/>
     </row>
     <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="11"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="18"/>
+      <c r="A33" s="6"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2528,15 +2112,15 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="12"/>
-      <c r="B34" s="13"/>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="20"/>
+    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="6"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
@@ -2666,11 +2250,6 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2678,6 +2257,11 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>